<commit_message>
Update Quiz und Risikoregister
</commit_message>
<xml_diff>
--- a/Risikoregister_KI-Beauftragte_Template.xlsx
+++ b/Risikoregister_KI-Beauftragte_Template.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7be0febd872b4f91/Dokumente/GitHub/KI_Schulungen_UNO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="11_0CB637C9CAA9701A0FEAE49338CF05F494D2DEC0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8683530E-B5E6-4EF6-88EA-341ADC5D67AB}"/>
+  <xr:revisionPtr revIDLastSave="151" documentId="11_0CB637C9CAA9701A0FEAE49338CF05F494D2DEC0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE29A253-0271-4D40-A88D-159011C9C12C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Anleitung" sheetId="1" r:id="rId1"/>
     <sheet name="KH-Beispiel" sheetId="2" r:id="rId2"/>
     <sheet name="Leeres Register" sheetId="3" r:id="rId3"/>
-    <sheet name="A-B-E-Skala" sheetId="4" r:id="rId4"/>
-    <sheet name="Listen" sheetId="5" r:id="rId5"/>
+    <sheet name="Visualisierung" sheetId="6" r:id="rId4"/>
+    <sheet name="A-B-E-Skala" sheetId="4" r:id="rId5"/>
+    <sheet name="Listen" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="192">
   <si>
     <t>Aufgabenbereich C: Risikoregister</t>
   </si>
@@ -598,13 +599,28 @@
   </si>
   <si>
     <t>Wert</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>UC</t>
+  </si>
+  <si>
+    <t>Name</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -715,6 +731,21 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -805,7 +836,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -859,22 +890,26 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1043,6 +1078,1113 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="4.1397467803571189E-2"/>
+          <c:y val="2.7894002789400279E-2"/>
+          <c:w val="0.93172861164375176"/>
+          <c:h val="0.84886106809870521"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:bubbleChart>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Visualisierung!$E$2:$E$4</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Doom-Loop-Bias der Trainingsdaten — Modell wurde 2020–2024 trainiert; "Normal" entspricht überlasteten Klinikbetrieben</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Automation Bias bei Radiologen — KI-Befunde werden mit zunehmender Trefferquote weniger kritisch geprüft</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Indien-Schnittstelle: Anbindung an externe Datenbank (10 Mio. CTs) ohne EU-Angemessenheitsbeschluss</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:pattFill prst="ltUpDiag">
+              <a:fgClr>
+                <a:schemeClr val="accent1"/>
+              </a:fgClr>
+              <a:bgClr>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="20000"/>
+                  <a:lumOff val="80000"/>
+                </a:schemeClr>
+              </a:bgClr>
+            </a:pattFill>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:alpha val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst>
+              <a:innerShdw blurRad="114300">
+                <a:schemeClr val="accent1">
+                  <a:alpha val="70000"/>
+                </a:schemeClr>
+              </a:innerShdw>
+            </a:effectLst>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="000000">
+                    <a:lumMod val="25000"/>
+                    <a:lumOff val="75000"/>
+                  </a:srgbClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-DE"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="1"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="wedgeRectCallout">
+                    <a:avLst/>
+                  </a:prstGeom>
+                  <a:noFill/>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                </c15:spPr>
+                <c15:showLeaderLines val="0"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Visualisierung!$F$2:$F$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Visualisierung!$G$2:$G$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:bubbleSize>
+            <c:numRef>
+              <c:f>Visualisierung!$H$2:$H$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>448</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>108</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:bubbleSize>
+          <c:bubble3D val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-C30E-406A-AEE2-6A1E943C0A60}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:bubbleScale val="100"/>
+        <c:showNegBubbles val="0"/>
+        <c:axId val="1287024992"/>
+        <c:axId val="1287021632"/>
+      </c:bubbleChart>
+      <c:valAx>
+        <c:axId val="1287024992"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="10"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Schadensschwere (B)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1287021632"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1287021632"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="10"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Wahrscheinlichkeit (A)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1287024992"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-DE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="270">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:effectRef>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:pattFill prst="ltUpDiag">
+        <a:fgClr>
+          <a:schemeClr val="phClr"/>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="phClr">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:bgClr>
+      </a:pattFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:alpha val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+      <a:effectLst>
+        <a:innerShdw blurRad="114300">
+          <a:schemeClr val="phClr">
+            <a:alpha val="70000"/>
+          </a:schemeClr>
+        </a:innerShdw>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:pattFill prst="ltUpDiag">
+        <a:fgClr>
+          <a:schemeClr val="phClr"/>
+        </a:fgClr>
+        <a:bgClr>
+          <a:schemeClr val="phClr">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:bgClr>
+      </a:pattFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:alpha val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+      <a:effectLst>
+        <a:innerShdw blurRad="114300">
+          <a:schemeClr val="phClr">
+            <a:alpha val="70000"/>
+          </a:schemeClr>
+        </a:innerShdw>
+      </a:effectLst>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="50000"/>
+        <a:lumOff val="50000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1800" b="1" kern="1200" cap="all" spc="150" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>83820</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>784860</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9D30F43-7630-8A6E-E1D9-F2734D615858}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1448,96 +2590,96 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
-      <c r="S1" s="26"/>
-      <c r="T1" s="26"/>
-      <c r="U1" s="26"/>
-      <c r="V1" s="26"/>
-      <c r="W1" s="26"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="29"/>
+      <c r="V1" s="29"/>
+      <c r="W1" s="29"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3" s="9"/>
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="30" t="s">
         <v>182</v>
       </c>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
       <c r="I3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="J3" s="31" t="s">
+      <c r="J3" s="30" t="s">
         <v>181</v>
       </c>
-      <c r="K3" s="26"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
       <c r="O3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="P3" s="31" t="s">
+      <c r="P3" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="Q3" s="26"/>
-      <c r="R3" s="26"/>
-      <c r="S3" s="26"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="29"/>
     </row>
     <row r="5" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="27" t="s">
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="27" t="s">
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="29"/>
-      <c r="O5" s="27" t="s">
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="26"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="P5" s="28"/>
-      <c r="Q5" s="29"/>
-      <c r="R5" s="27" t="s">
+      <c r="P5" s="26"/>
+      <c r="Q5" s="27"/>
+      <c r="R5" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="S5" s="28"/>
-      <c r="T5" s="28"/>
-      <c r="U5" s="28"/>
-      <c r="V5" s="29"/>
+      <c r="S5" s="26"/>
+      <c r="T5" s="26"/>
+      <c r="U5" s="26"/>
+      <c r="V5" s="27"/>
       <c r="W5" s="3" t="s">
         <v>10</v>
       </c>
@@ -1651,17 +2793,17 @@
         <v>44</v>
       </c>
       <c r="J7" s="12">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K7" s="12">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L7" s="12">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M7" s="12">
         <f t="shared" ref="M7:M11" si="0">IF(COUNTA(J7:L7)=3,J7*K7*L7,"")</f>
-        <v>336</v>
+        <v>24</v>
       </c>
       <c r="N7" s="13" t="s">
         <v>45</v>
@@ -1809,17 +2951,17 @@
         <v>74</v>
       </c>
       <c r="J9" s="12">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K9" s="12">
+        <v>2</v>
+      </c>
+      <c r="L9" s="12">
         <v>9</v>
-      </c>
-      <c r="L9" s="12">
-        <v>5</v>
       </c>
       <c r="M9" s="12">
         <f t="shared" si="0"/>
-        <v>180</v>
+        <v>108</v>
       </c>
       <c r="N9" s="13" t="s">
         <v>75</v>
@@ -1943,10 +3085,10 @@
       <c r="D13" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="E13" s="25" t="s">
+      <c r="E13" s="31" t="s">
         <v>85</v>
       </c>
-      <c r="F13" s="26"/>
+      <c r="F13" s="29"/>
       <c r="G13" s="17" t="s">
         <v>86</v>
       </c>
@@ -1955,32 +3097,32 @@
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="32" t="s">
         <v>88</v>
       </c>
-      <c r="B14" s="26"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="26"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="29"/>
+      <c r="G14" s="29"/>
+      <c r="H14" s="29"/>
+      <c r="I14" s="29"/>
+      <c r="J14" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A14:J14"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="B3:H3"/>
     <mergeCell ref="O5:Q5"/>
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="J3:N3"/>
     <mergeCell ref="J5:N5"/>
     <mergeCell ref="P3:S3"/>
     <mergeCell ref="R5:V5"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A14:J14"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="B3:H3"/>
   </mergeCells>
   <conditionalFormatting sqref="M7:M11">
     <cfRule type="cellIs" dxfId="11" priority="2" operator="lessThan">
@@ -2072,31 +3214,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
-      <c r="Q1" s="26"/>
-      <c r="R1" s="26"/>
-      <c r="S1" s="26"/>
-      <c r="T1" s="26"/>
-      <c r="U1" s="26"/>
-      <c r="V1" s="26"/>
-      <c r="W1" s="26"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="29"/>
+      <c r="Q1" s="29"/>
+      <c r="R1" s="29"/>
+      <c r="S1" s="29"/>
+      <c r="T1" s="29"/>
+      <c r="U1" s="29"/>
+      <c r="V1" s="29"/>
+      <c r="W1" s="29"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3" s="9"/>
@@ -2112,52 +3254,52 @@
         <v>179</v>
       </c>
       <c r="I3" s="24"/>
-      <c r="J3" s="31"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
+      <c r="J3" s="30"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
       <c r="O3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="P3" s="31"/>
-      <c r="Q3" s="26"/>
-      <c r="R3" s="26"/>
-      <c r="S3" s="26"/>
+      <c r="P3" s="30"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="29"/>
     </row>
     <row r="5" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="27" t="s">
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="27" t="s">
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="29"/>
-      <c r="O5" s="27" t="s">
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="26"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="P5" s="28"/>
-      <c r="Q5" s="29"/>
-      <c r="R5" s="27" t="s">
+      <c r="P5" s="26"/>
+      <c r="Q5" s="27"/>
+      <c r="R5" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="S5" s="28"/>
-      <c r="T5" s="28"/>
-      <c r="U5" s="28"/>
-      <c r="V5" s="29"/>
+      <c r="S5" s="26"/>
+      <c r="T5" s="26"/>
+      <c r="U5" s="26"/>
+      <c r="V5" s="27"/>
       <c r="W5" s="3" t="s">
         <v>10</v>
       </c>
@@ -2390,6 +3532,129 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98EC6ED1-D120-465B-B739-F578E23E3203}">
+  <dimension ref="D1:H9"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="2.33203125" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" style="36"/>
+    <col min="5" max="5" width="22.109375" style="36" customWidth="1"/>
+    <col min="6" max="8" width="8.6640625" style="36"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="4:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D1" s="35" t="s">
+        <v>190</v>
+      </c>
+      <c r="E1" s="35" t="s">
+        <v>191</v>
+      </c>
+      <c r="F1" s="35" t="s">
+        <v>187</v>
+      </c>
+      <c r="G1" s="35" t="s">
+        <v>188</v>
+      </c>
+      <c r="H1" s="35" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="2" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D2" s="36">
+        <f>+'KH-Beispiel'!A7</f>
+        <v>1</v>
+      </c>
+      <c r="E2" s="36" t="str">
+        <f>+'KH-Beispiel'!F7</f>
+        <v>Doom-Loop-Bias der Trainingsdaten — Modell wurde 2020–2024 trainiert; "Normal" entspricht überlasteten Klinikbetrieben</v>
+      </c>
+      <c r="F2" s="36">
+        <f>+'KH-Beispiel'!J7</f>
+        <v>2</v>
+      </c>
+      <c r="G2" s="36">
+        <f>+'KH-Beispiel'!K7</f>
+        <v>4</v>
+      </c>
+      <c r="H2" s="36">
+        <f>+'KH-Beispiel'!M7</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D3" s="36">
+        <f>+'KH-Beispiel'!A8</f>
+        <v>2</v>
+      </c>
+      <c r="E3" s="36" t="str">
+        <f>+'KH-Beispiel'!F8</f>
+        <v>Automation Bias bei Radiologen — KI-Befunde werden mit zunehmender Trefferquote weniger kritisch geprüft</v>
+      </c>
+      <c r="F3" s="36">
+        <f>+'KH-Beispiel'!J8</f>
+        <v>7</v>
+      </c>
+      <c r="G3" s="36">
+        <f>+'KH-Beispiel'!K8</f>
+        <v>8</v>
+      </c>
+      <c r="H3" s="36">
+        <f>+'KH-Beispiel'!M8</f>
+        <v>448</v>
+      </c>
+    </row>
+    <row r="4" spans="4:8" x14ac:dyDescent="0.3">
+      <c r="D4" s="36">
+        <f>+'KH-Beispiel'!A9</f>
+        <v>3</v>
+      </c>
+      <c r="E4" s="36" t="str">
+        <f>+'KH-Beispiel'!F9</f>
+        <v>Indien-Schnittstelle: Anbindung an externe Datenbank (10 Mio. CTs) ohne EU-Angemessenheitsbeschluss</v>
+      </c>
+      <c r="F4" s="36">
+        <f>+'KH-Beispiel'!J9</f>
+        <v>6</v>
+      </c>
+      <c r="G4" s="36">
+        <f>+'KH-Beispiel'!K9</f>
+        <v>2</v>
+      </c>
+      <c r="H4" s="36">
+        <f>+'KH-Beispiel'!M9</f>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="5" spans="4:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D5" s="36">
+        <f>+'KH-Beispiel'!A10</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="36">
+        <f>+'KH-Beispiel'!J10</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="36">
+        <f>+'KH-Beispiel'!K10</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="36" t="str">
+        <f>+'KH-Beispiel'!M10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="4:8" ht="49.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="4:8" ht="94.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="4:8" ht="94.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="4:8" ht="94.5" customHeight="1" x14ac:dyDescent="0.3"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2400,20 +3665,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="28" t="s">
         <v>124</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="32" t="s">
         <v>125</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
     </row>
     <row r="4" spans="1:4" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
@@ -2573,9 +3838,9 @@
       <c r="A17" s="34" t="s">
         <v>160</v>
       </c>
-      <c r="B17" s="26"/>
-      <c r="C17" s="26"/>
-      <c r="D17" s="26"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2588,7 +3853,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>